<commit_message>
Lote 6: corregir descripción NV11D/NV11P/NV11R según imágenes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bWxU7GBEhMMMrCBgBXSaR
</commit_message>
<xml_diff>
--- a/PRODUCTOS_RAPPI/ESTRUCTURA_RAPPI_LOTE6.xlsx
+++ b/PRODUCTOS_RAPPI/ESTRUCTURA_RAPPI_LOTE6.xlsx
@@ -9255,8 +9255,8 @@
       </c>
       <c r="C301" s="5" t="inlineStr">
         <is>
-          <t>- Flor navideña artificial de 30 cm en plástico, color palo de rosa
-- Apariencia realista con textura delicada y brillo duradero
+          <t>- Ramillete navideño decorativo de 30 cm con acabado escarchado en purpurina, color palo de rosa
+- Ramitas finas tipo ciprés que reflejan la luz y dan un brillo elegante
 - Se integra fácilmente al árbol de Navidad sin pasos complicados
 - Resistente: mantiene su color y forma por mucho tiempo
 - Ideal para árbol, decoración del hogar, fiestas y bodas</t>
@@ -9284,8 +9284,8 @@
       </c>
       <c r="C302" s="5" t="inlineStr">
         <is>
-          <t>- Flor navideña artificial de 30 cm en plástico, color rojo
-- Apariencia realista con textura delicada y brillo duradero
+          <t>- Ramillete navideño decorativo de 30 cm con acabado escarchado en purpurina, color rojo
+- Ramitas finas tipo ciprés que reflejan la luz y dan un brillo elegante
 - Se integra fácilmente al árbol de Navidad sin pasos complicados
 - Resistente: mantiene su color y forma por mucho tiempo
 - Ideal para árbol, decoración del hogar, fiestas y bodas</t>
@@ -9313,8 +9313,8 @@
       </c>
       <c r="C303" s="5" t="inlineStr">
         <is>
-          <t>- Flor navideña artificial de 30 cm en plástico, color dorado
-- Apariencia realista con textura delicada y brillo duradero
+          <t>- Ramillete navideño decorativo de 30 cm con acabado escarchado en purpurina, color dorado
+- Ramitas finas tipo ciprés que reflejan la luz y dan un brillo elegante
 - Se integra fácilmente al árbol de Navidad sin pasos complicados
 - Resistente: mantiene su color y forma por mucho tiempo
 - Ideal para árbol, decoración del hogar, fiestas y bodas</t>

</xml_diff>